<commit_message>
fix(productos): Kit de Tareas (representante) — 4 defectos vivos en producción corregidos con el motor 2.4: mensaje de la DV coherente con el contador, «Total facturado = efectivo contado − fondo + tarjetas + otros», 08 sin contradecirse sobre el marco del día, TPV del 09 como comprobación (no segundo encendido), frase honesta de niveles y calendario BONUS-02 editable; diff contra producción 177 = 26 valor + 33 DV + 26 alturas + 92 locked (igual al firmado)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/kit-tareas/01-apertura-cierre.xlsx
+++ b/astro-site/public/dl/kit-tareas/01-apertura-cierre.xlsx
@@ -899,6 +899,7 @@
         </is>
       </c>
     </row>
+    <row r="24"/>
     <row r="25" ht="32" customHeight="1">
       <c r="B25" s="41" t="inlineStr">
         <is>
@@ -913,6 +914,7 @@
         </is>
       </c>
     </row>
+    <row r="27"/>
     <row r="28" ht="18" customHeight="1">
       <c r="B28" s="40" t="inlineStr">
         <is>
@@ -920,6 +922,7 @@
         </is>
       </c>
     </row>
+    <row r="29"/>
     <row r="30" ht="32" customHeight="1">
       <c r="B30" s="41" t="inlineStr">
         <is>
@@ -934,6 +937,7 @@
         </is>
       </c>
     </row>
+    <row r="32"/>
     <row r="33" ht="18" customHeight="1">
       <c r="B33" s="40" t="inlineStr">
         <is>
@@ -941,10 +945,11 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="32" customHeight="1">
+    <row r="34"/>
+    <row r="35" ht="16" customHeight="1">
       <c r="B35" s="41" t="inlineStr">
         <is>
-          <t>▸ 08-apertura-cierre-negocio.xlsx — checklist del LOCAL completo: es el MARCO del día (accesos, luces, clima, terraza).</t>
+          <t>▸ 08-apertura-cierre-negocio.xlsx — checklist del LOCAL completo: es el MARCO del día.</t>
         </is>
       </c>
     </row>
@@ -962,10 +967,10 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="16" customHeight="1">
+    <row r="38" ht="48" customHeight="1">
       <c r="B38" s="41" t="inlineStr">
         <is>
-          <t>▸ Orden de uso: local → áreas → caja. No se duplican: cada uno cubre un nivel.</t>
+          <t>▸ Orden de uso: local → áreas → caja. Cada fichero cubre un nivel: el de negocio marca el HITO (encender, abrir, cerrar), el de áreas detalla CÓMO se hace en cada zona y el de caja lleva el DINERO. Si una tarea aparece en dos, es a propósito: una es el hito y la otra el detalle.</t>
         </is>
       </c>
     </row>
@@ -976,6 +981,7 @@
         </is>
       </c>
     </row>
+    <row r="40"/>
     <row r="41" ht="18" customHeight="1">
       <c r="B41" s="40" t="inlineStr">
         <is>
@@ -983,6 +989,7 @@
         </is>
       </c>
     </row>
+    <row r="42"/>
     <row r="43" ht="35" customHeight="1">
       <c r="B43" s="40" t="inlineStr">
         <is>
@@ -997,6 +1004,7 @@
         </is>
       </c>
     </row>
+    <row r="45"/>
     <row r="46" ht="18" customHeight="1">
       <c r="B46" s="40" t="inlineStr">
         <is>
@@ -2135,7 +2143,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F6 F7 F8 F9 F10 F13 F14 F15 F16 F17 F18 F21 F22 F23 F24 F27 F28 F29 F30 F33 F34 F35 F36 F37 F38 F39 F42 F43 F44 F45 F46 F47 F48 F49 F50" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Marca no válida" error="Usa el desplegable: ✓ (hecha), — (no hecha) o N/A (no aplica). Las marcadas N/A o — salen del total." type="list" errorStyle="stop">
+    <dataValidation sqref="F6 F7 F8 F9 F10 F13 F14 F15 F16 F17 F18 F21 F22 F23 F24 F27 F28 F29 F30 F33 F34 F35 F36 F37 F38 F39 F42 F43 F44 F45 F46 F47 F48 F49 F50" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Marca no válida" error="Usa el desplegable: ✓, — o N/A. N/A = no aplica, sale del total; — = no hecha, cuenta como pendiente." type="list" errorStyle="stop">
       <formula1>"✓,—,N/A"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2159,7 +2167,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2880,11 +2888,6 @@
         </is>
       </c>
     </row>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="0"/>
   <mergeCells count="9">
@@ -2894,9 +2897,9 @@
     <mergeCell ref="A14:G14"/>
     <mergeCell ref="A5:G5"/>
     <mergeCell ref="A21:G21"/>
+    <mergeCell ref="A29:G29"/>
     <mergeCell ref="A36:C36"/>
     <mergeCell ref="F38:G38"/>
-    <mergeCell ref="A29:G29"/>
   </mergeCells>
   <conditionalFormatting sqref="A5:G34">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -2904,7 +2907,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F6 F7 F8 F9 F10 F11 F12 F15 F16 F17 F18 F19 F22 F23 F24 F25 F26 F27 F28 F30 F31 F32 F33 F34" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Marca no válida" error="Usa el desplegable: ✓ (hecha), — (no hecha) o N/A (no aplica). Las marcadas N/A o — salen del total." type="list" errorStyle="stop">
+    <dataValidation sqref="F6 F7 F8 F9 F10 F11 F12 F15 F16 F17 F18 F19 F22 F23 F24 F25 F26 F27 F28 F30 F31 F32 F33 F34" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Marca no válida" error="Usa el desplegable: ✓, — o N/A. N/A = no aplica, sale del total; — = no hecha, cuenta como pendiente." type="list" errorStyle="stop">
       <formula1>"✓,—,N/A"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3578,9 +3581,9 @@
   <mergeCells count="8">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A32:C32"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="F34:G34"/>
     <mergeCell ref="A14:G14"/>
-    <mergeCell ref="F34:G34"/>
-    <mergeCell ref="A2:G2"/>
     <mergeCell ref="B34:D34"/>
     <mergeCell ref="A5:G5"/>
     <mergeCell ref="A21:G21"/>
@@ -3591,7 +3594,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F6 F7 F8 F9 F10 F11 F12 F15 F16 F17 F18 F19 F22 F23 F24 F25 F26 F27 F28 F29 F30" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Marca no válida" error="Usa el desplegable: ✓ (hecha), — (no hecha) o N/A (no aplica). Las marcadas N/A o — salen del total." type="list" errorStyle="stop">
+    <dataValidation sqref="F6 F7 F8 F9 F10 F11 F12 F15 F16 F17 F18 F19 F22 F23 F24 F25 F26 F27 F28 F29 F30" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Marca no válida" error="Usa el desplegable: ✓, — o N/A. N/A = no aplica, sale del total; — = no hecha, cuenta como pendiente." type="list" errorStyle="stop">
       <formula1>"✓,—,N/A"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4531,11 +4534,11 @@
     <mergeCell ref="F45:G45"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="B45:D45"/>
+    <mergeCell ref="A2:G2"/>
     <mergeCell ref="A14:G14"/>
-    <mergeCell ref="A2:G2"/>
     <mergeCell ref="A30:G30"/>
+    <mergeCell ref="A43:C43"/>
     <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A43:C43"/>
     <mergeCell ref="A22:G22"/>
   </mergeCells>
   <conditionalFormatting sqref="A5:G41">
@@ -4544,7 +4547,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F6 F7 F8 F9 F10 F11 F12 F15 F16 F17 F18 F19 F20 F23 F24 F25 F26 F27 F28 F31 F32 F33 F34 F35 F36 F37 F38 F39 F40 F41" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Marca no válida" error="Usa el desplegable: ✓ (hecha), — (no hecha) o N/A (no aplica). Las marcadas N/A o — salen del total." type="list" errorStyle="stop">
+    <dataValidation sqref="F6 F7 F8 F9 F10 F11 F12 F15 F16 F17 F18 F19 F20 F23 F24 F25 F26 F27 F28 F31 F32 F33 F34 F35 F36 F37 F38 F39 F40 F41" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Marca no válida" error="Usa el desplegable: ✓, — o N/A. N/A = no aplica, sale del total; — = no hecha, cuenta como pendiente." type="list" errorStyle="stop">
       <formula1>"✓,—,N/A"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4568,7 +4571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5073,17 +5076,6 @@
         </is>
       </c>
     </row>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="0"/>
   <mergeCells count="9">
@@ -5103,7 +5095,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F6 F7 F8 F9 F10 F11 F14 F15 F16 F17 F18 F20 F22 F23 F24 F25 F26" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Marca no válida" error="Usa el desplegable: ✓ (hecha), — (no hecha) o N/A (no aplica). Las marcadas N/A o — salen del total." type="list" errorStyle="stop">
+    <dataValidation sqref="F6 F7 F8 F9 F10 F11 F14 F15 F16 F17 F18 F20 F22 F23 F24 F25 F26" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Marca no válida" error="Usa el desplegable: ✓, — o N/A. N/A = no aplica, sale del total; — = no hecha, cuenta como pendiente." type="list" errorStyle="stop">
       <formula1>"✓,—,N/A"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5659,7 +5651,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F6 F7 F8 F9 F10 F11 F14 F15 F16 F17 F18 F19 F20 F21 F22 F23 F24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Marca no válida" error="Usa el desplegable: ✓ (hecha), — (no hecha) o N/A (no aplica). Las marcadas N/A o — salen del total." type="list" errorStyle="stop">
+    <dataValidation sqref="F6 F7 F8 F9 F10 F11 F14 F15 F16 F17 F18 F19 F20 F21 F22 F23 F24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Marca no válida" error="Usa el desplegable: ✓, — o N/A. N/A = no aplica, sale del total; — = no hecha, cuenta como pendiente." type="list" errorStyle="stop">
       <formula1>"✓,—,N/A"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>